<commit_message>
update with 0.5mm Glaston line capability
</commit_message>
<xml_diff>
--- a/AlpenGlass max sizing data.xlsx
+++ b/AlpenGlass max sizing data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alpencustomersupport.sharepoint.com/sites/GlassProgram2/Shared Documents/AlpenGlass Channel/00. Product Info/AlpenGlass Catalog &amp; Pricing/Catalog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{75EA31A8-BFAF-4EC6-93D9-1890CDCF103F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA7CA4FC-C5DE-4A91-BE25-87A02B54C08B}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{75EA31A8-BFAF-4EC6-93D9-1890CDCF103F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85FECB3E-7EED-450E-B3AC-B852AB0767F9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3B798C6C-F77F-4AFD-8CF8-D88FE96A59C4}"/>
+    <workbookView xWindow="-28920" yWindow="-3225" windowWidth="29040" windowHeight="15720" xr2:uid="{3B798C6C-F77F-4AFD-8CF8-D88FE96A59C4}"/>
   </bookViews>
   <sheets>
     <sheet name="tempered" sheetId="1" r:id="rId1"/>
@@ -1452,10 +1452,10 @@
       <c r="J5" s="1"/>
       <c r="K5" s="7">
         <f>Table1[[#This Row],[Technical_limit_longedge_inches]]*Table1[[#This Row],[Technical_limit_shortedge_inches]]/144</f>
-        <v>40.833333333333336</v>
+        <v>49.583333333333336</v>
       </c>
       <c r="L5" s="1">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="M5" s="1">
         <v>60</v>
@@ -1575,10 +1575,10 @@
       <c r="J8" s="1"/>
       <c r="K8" s="7">
         <f>Table1[[#This Row],[Technical_limit_longedge_inches]]*Table1[[#This Row],[Technical_limit_shortedge_inches]]/144</f>
-        <v>49</v>
+        <v>49.5</v>
       </c>
       <c r="L8" s="1">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M8" s="1">
         <v>72</v>
@@ -1616,10 +1616,10 @@
       <c r="J9" s="1"/>
       <c r="K9" s="7">
         <f>Table1[[#This Row],[Technical_limit_longedge_inches]]*Table1[[#This Row],[Technical_limit_shortedge_inches]]/144</f>
-        <v>49.5</v>
+        <v>59.5</v>
       </c>
       <c r="L9" s="1">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="M9" s="1">
         <v>72</v>
@@ -2370,26 +2370,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="891be25f-b2fc-4437-ac28-9b63a2a6eb24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010099EB33AB64FFCD4AA4628371E25A8D85" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="796bff8b10082fc3cc57856a82f602f3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="891be25f-b2fc-4437-ac28-9b63a2a6eb24" xmlns:ns3="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="649ae9b12cda5c629f22bcf27b9f706f" ns2:_="" ns3:_="">
     <xsd:import namespace="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
@@ -2590,26 +2570,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{555DF2C4-5AEB-4283-88B9-E34AFF223611}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
-    <ds:schemaRef ds:uri="63da1fdb-95da-4a03-a2ac-dcaabea38ae8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EAC9F8B-5315-457E-A63B-9DC144062226}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="891be25f-b2fc-4437-ac28-9b63a2a6eb24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1BFF9EE-31C6-459B-B806-749437464102}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2626,4 +2607,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EAC9F8B-5315-457E-A63B-9DC144062226}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{555DF2C4-5AEB-4283-88B9-E34AFF223611}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
+    <ds:schemaRef ds:uri="63da1fdb-95da-4a03-a2ac-dcaabea38ae8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
correct 6mm.0.5mm/6mm custom size rang
with glaston capability
</commit_message>
<xml_diff>
--- a/AlpenGlass max sizing data.xlsx
+++ b/AlpenGlass max sizing data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alpencustomersupport.sharepoint.com/sites/GlassProgram2/Shared Documents/AlpenGlass Channel/00. Product Info/AlpenGlass Catalog &amp; Pricing/Catalog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{75EA31A8-BFAF-4EC6-93D9-1890CDCF103F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85FECB3E-7EED-450E-B3AC-B852AB0767F9}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{75EA31A8-BFAF-4EC6-93D9-1890CDCF103F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E526A25-A191-45F0-9FAE-B4FAC865ACE2}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-3225" windowWidth="29040" windowHeight="15720" xr2:uid="{3B798C6C-F77F-4AFD-8CF8-D88FE96A59C4}"/>
   </bookViews>
@@ -1575,10 +1575,10 @@
       <c r="J8" s="1"/>
       <c r="K8" s="7">
         <f>Table1[[#This Row],[Technical_limit_longedge_inches]]*Table1[[#This Row],[Technical_limit_shortedge_inches]]/144</f>
-        <v>49.5</v>
+        <v>59.5</v>
       </c>
       <c r="L8" s="1">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="M8" s="1">
         <v>72</v>
@@ -1616,10 +1616,10 @@
       <c r="J9" s="1"/>
       <c r="K9" s="7">
         <f>Table1[[#This Row],[Technical_limit_longedge_inches]]*Table1[[#This Row],[Technical_limit_shortedge_inches]]/144</f>
-        <v>59.5</v>
+        <v>49.5</v>
       </c>
       <c r="L9" s="1">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="M9" s="1">
         <v>72</v>
@@ -2370,6 +2370,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="891be25f-b2fc-4437-ac28-9b63a2a6eb24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010099EB33AB64FFCD4AA4628371E25A8D85" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="796bff8b10082fc3cc57856a82f602f3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="891be25f-b2fc-4437-ac28-9b63a2a6eb24" xmlns:ns3="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="649ae9b12cda5c629f22bcf27b9f706f" ns2:_="" ns3:_="">
     <xsd:import namespace="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
@@ -2570,27 +2590,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{555DF2C4-5AEB-4283-88B9-E34AFF223611}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
+    <ds:schemaRef ds:uri="63da1fdb-95da-4a03-a2ac-dcaabea38ae8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="891be25f-b2fc-4437-ac28-9b63a2a6eb24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="63da1fdb-95da-4a03-a2ac-dcaabea38ae8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EAC9F8B-5315-457E-A63B-9DC144062226}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1BFF9EE-31C6-459B-B806-749437464102}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2607,23 +2626,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EAC9F8B-5315-457E-A63B-9DC144062226}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{555DF2C4-5AEB-4283-88B9-E34AFF223611}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="891be25f-b2fc-4437-ac28-9b63a2a6eb24"/>
-    <ds:schemaRef ds:uri="63da1fdb-95da-4a03-a2ac-dcaabea38ae8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>